<commit_message>
Update berita 2026-08-04 07:29 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-08-02.xlsx
+++ b/data/berita_antara_2026-08-02.xlsx
@@ -987,33 +987,33 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>politik</t>
+          <t>photo</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>4 contoh sambutan ketua panitia 17 Agustus 2026 singkat, formal, dan penuh makna</t>
+          <t>Melihat balap babi di Amerika</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 11:04:26 +0700</t>
+          <t>Sun, 02 Aug 2026 17:06:31 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Peringatan HUT ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026 menjadi momentum bagi masyarakat untuk ...</t>
+          <t>Sejumlah babi berlomba dalam kompetisi balap babi pada Orange County Fair di Costa Mesa, California, Amerika Serikat, (1/8/2026). ANTARA FOTO/Xinhua/Qiu Chen/sgd</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676415/4-contoh-sambutan-ketua-panitia-17-agustus-2026-singkat-formal-dan-penuh-makna</t>
+          <t>https://www.antaranews.com/foto/5676656/melihat-balap-babi-di-amerika</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2025/08/18/lomba-memerihakan-hut-kemerdekaan-ri-di-ciamis-2602537.jpg</t>
+          <t>https://cdn.antaranews.com/cache/255x170/2026/08/02/XxjpbeE000086_20260802_PEPFN0A001.jpg</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1030,28 +1030,28 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Cara daftar Upacara 17 Agustus 2026 di Istana Merdeka, simak syarat dan jadwalnya</t>
+          <t>4 contoh sambutan ketua panitia 17 Agustus 2026 singkat, formal, dan penuh makna</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 10:59:29 +0700</t>
+          <t>Sun, 02 Aug 2026 11:04:26 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Pemerintah belum mengumumkan jadwal resmi pembukaan pendaftaran peserta upacara peringatan HUT ke-81 Kemerdekaan ...</t>
+          <t>Peringatan HUT ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026 menjadi momentum bagi masyarakat untuk ...</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676408/cara-daftar-upacara-17-agustus-2026-di-istana-merdeka-simak-syarat-dan-jadwalnya</t>
+          <t>https://www.antaranews.com/berita/5676415/4-contoh-sambutan-ketua-panitia-17-agustus-2026-singkat-formal-dan-penuh-makna</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/02/Upacara-Prasetya-Perwira-TNI-POLRI-22072026-gp-2.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/08/18/lomba-memerihakan-hut-kemerdekaan-ri-di-ciamis-2602537.jpg</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1063,33 +1063,33 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>humaniora</t>
+          <t>politik</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Cara mencairkan bansos PKH dan BPNT Agustus 2026 lewat bank dan kantor pos</t>
+          <t>Cara daftar Upacara 17 Agustus 2026 di Istana Merdeka, simak syarat dan jadwalnya</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 10:51:29 +0700</t>
+          <t>Sun, 02 Aug 2026 10:59:29 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Penyaluran bantuan sosial Program Keluarga Harapan (PKH) dan Bantuan Pangan Non Tunai (BPNT) periode Agustus 2026 ...</t>
+          <t>Pemerintah belum mengumumkan jadwal resmi pembukaan pendaftaran peserta upacara peringatan HUT ke-81 Kemerdekaan ...</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676407/cara-mencairkan-bansos-pkh-dan-bpnt-agustus-2026-lewat-bank-dan-kantor-pos</t>
+          <t>https://www.antaranews.com/berita/5676408/cara-daftar-upacara-17-agustus-2026-di-istana-merdeka-simak-syarat-dan-jadwalnya</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/03/27/IMG_20260327_142333.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/02/Upacara-Prasetya-Perwira-TNI-POLRI-22072026-gp-2.jpg</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1106,28 +1106,28 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>NIK tidak ditemukan saat cek bansos? Ini 6 penyebab dan cara mengatasinya</t>
+          <t>Cara mencairkan bansos PKH dan BPNT Agustus 2026 lewat bank dan kantor pos</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 10:43:03 +0700</t>
+          <t>Sun, 02 Aug 2026 10:51:29 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Sebagian masyarakat masih mengalami kendala saat mengecek status penerima bantuan sosial (bansos), salah satunya muncul ...</t>
+          <t>Penyaluran bantuan sosial Program Keluarga Harapan (PKH) dan Bantuan Pangan Non Tunai (BPNT) periode Agustus 2026 ...</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676401/nik-tidak-ditemukan-saat-cek-bansos-ini-6-penyebab-dan-cara-mengatasinya</t>
+          <t>https://www.antaranews.com/berita/5676407/cara-mencairkan-bansos-pkh-dan-bpnt-agustus-2026-lewat-bank-dan-kantor-pos</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/07/bansos-ngawi-1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/27/IMG_20260327_142333.jpg</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1139,33 +1139,33 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>lifestyle</t>
+          <t>humaniora</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Waspada! Ini ciri-ciri kalau mata Anda mulai minus</t>
+          <t>NIK tidak ditemukan saat cek bansos? Ini 6 penyebab dan cara mengatasinya</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 23:27:26 +0700</t>
+          <t>Sun, 02 Aug 2026 10:43:03 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Miopi atau mata minus adalah gangguan refraksi yang menyebabkan seseorang kesulitan melihat benda yang berada di ...</t>
+          <t>Sebagian masyarakat masih mengalami kendala saat mengecek status penerima bantuan sosial (bansos), salah satunya muncul ...</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676920/waspada-ini-ciri-ciri-kalau-mata-anda-mulai-minus</t>
+          <t>https://www.antaranews.com/berita/5676401/nik-tidak-ditemukan-saat-cek-bansos-ini-6-penyebab-dan-cara-mengatasinya</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2024/03/27/antarafoto-safari-kesehatan-2024-270324-nhw-4.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/07/bansos-ngawi-1.jpeg</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1182,28 +1182,28 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Kenali ciri-ciri kecanduan PMO dan bagaimana cara mengatasinya</t>
+          <t>Waspada! Ini ciri-ciri kalau mata Anda mulai minus</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 23:24:09 +0700</t>
+          <t>Sun, 02 Aug 2026 23:27:26 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Kecanduan PMO atau Pornography, Masturbation, Orgasm menjadi salah satu topik yang semakin banyak diperbincangkan, ...</t>
+          <t>Miopi atau mata minus adalah gangguan refraksi yang menyebabkan seseorang kesulitan melihat benda yang berada di ...</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676919/kenali-ciri-ciri-kecanduan-pmo-dan-bagaimana-cara-mengatasinya</t>
+          <t>https://www.antaranews.com/berita/5676920/waspada-ini-ciri-ciri-kalau-mata-anda-mulai-minus</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/02/ilustrasi-konten-berbau-pornografi.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/03/27/antarafoto-safari-kesehatan-2024-270324-nhw-4.jpg</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1220,28 +1220,28 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Suka mual saat olahraga? Ini penyebab dan cara atasinya</t>
+          <t>Kenali ciri-ciri kecanduan PMO dan bagaimana cara mengatasinya</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 23:19:36 +0700</t>
+          <t>Sun, 02 Aug 2026 23:24:09 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Olahraga seharusnya membuat tubuh terasa lebih segar dan bugar. Namun, sebagian orang justru mengalami mual saat sedang ...</t>
+          <t>Kecanduan PMO atau Pornography, Masturbation, Orgasm menjadi salah satu topik yang semakin banyak diperbincangkan, ...</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676912/suka-mual-saat-olahraga-ini-penyebab-dan-cara-atasinya</t>
+          <t>https://www.antaranews.com/berita/5676919/kenali-ciri-ciri-kecanduan-pmo-dan-bagaimana-cara-mengatasinya</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2020/05/02/stretching-498256_1280.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/02/ilustrasi-konten-berbau-pornografi.jpg</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1258,28 +1258,28 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>10 Makanan yang bagus untuk bulu kucing agar tetap lebat dan berkilau</t>
+          <t>Suka mual saat olahraga? Ini penyebab dan cara atasinya</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 22:58:56 +0700</t>
+          <t>Sun, 02 Aug 2026 23:19:36 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Bulu yang lebat, halus, dan berkilau menjadi salah satu tanda bahwa kucing berada dalam kondisi sehat. Selain ...</t>
+          <t>Olahraga seharusnya membuat tubuh terasa lebih segar dan bugar. Namun, sebagian orang justru mengalami mual saat sedang ...</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676901/10-makanan-yang-bagus-untuk-bulu-kucing-agar-tetap-lebat-dan-berkilau</t>
+          <t>https://www.antaranews.com/berita/5676912/suka-mual-saat-olahraga-ini-penyebab-dan-cara-atasinya</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2019/08/16/IMG_1785.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2020/05/02/stretching-498256_1280.jpg</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1296,28 +1296,28 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Inilah 10 penyebab kucing tidak mau makan dan cara atasinya</t>
+          <t>10 Makanan yang bagus untuk bulu kucing agar tetap lebat dan berkilau</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 22:55:13 +0700</t>
+          <t>Sun, 02 Aug 2026 22:58:56 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Kucing yang tiba-tiba tidak mau makan tentu membuat pemiliknya khawatir. Pasalnya, nafsu makan merupakan salah satu ...</t>
+          <t>Bulu yang lebat, halus, dan berkilau menjadi salah satu tanda bahwa kucing berada dalam kondisi sehat. Selain ...</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676893/inilah-10-penyebab-kucing-tidak-mau-makan-dan-cara-atasinya</t>
+          <t>https://www.antaranews.com/berita/5676901/10-makanan-yang-bagus-untuk-bulu-kucing-agar-tetap-lebat-dan-berkilau</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2021/08/08/IMG_20210808_073426-01.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2019/08/16/IMG_1785.jpg</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1334,28 +1334,28 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Apa Itu digital detox? Manfaat, cara memulai, dan dampaknya bagi kesehatan mental</t>
+          <t>Inilah 10 penyebab kucing tidak mau makan dan cara atasinya</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 11:23:42 +0700</t>
+          <t>Sun, 02 Aug 2026 22:55:13 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Digital detox semakin banyak dibicarakan seiring meningkatnya kesadaran masyarakat terhadap dampak penggunaan gadget ...</t>
+          <t>Kucing yang tiba-tiba tidak mau makan tentu membuat pemiliknya khawatir. Pasalnya, nafsu makan merupakan salah satu ...</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676429/apa-itu-digital-detox-manfaat-cara-memulai-dan-dampaknya-bagi-kesehatan-mental</t>
+          <t>https://www.antaranews.com/berita/5676893/inilah-10-penyebab-kucing-tidak-mau-makan-dan-cara-atasinya</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2018/02/handphone.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2021/08/08/IMG_20210808_073426-01.jpeg</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1372,28 +1372,28 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>7 manfaat baby oil untuk wajah serta cara menggunakannya dengan aman</t>
+          <t>Apa Itu digital detox? Manfaat, cara memulai, dan dampaknya bagi kesehatan mental</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 11:14:29 +0700</t>
+          <t>Sun, 02 Aug 2026 11:23:42 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Baby oil tidak hanya digunakan untuk perawatan kulit bayi, tetapi juga kerap dimanfaatkan sebagai bagian dari rutinitas ...</t>
+          <t>Digital detox semakin banyak dibicarakan seiring meningkatnya kesadaran masyarakat terhadap dampak penggunaan gadget ...</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676420/7-manfaat-baby-oil-untuk-wajah-serta-cara-menggunakannya-dengan-aman</t>
+          <t>https://www.antaranews.com/berita/5676429/apa-itu-digital-detox-manfaat-cara-memulai-dan-dampaknya-bagi-kesehatan-mental</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/04/23/Tua.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2018/02/handphone.jpg</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1410,28 +1410,28 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>20 ide hadiah lomba 17 Agustus 2026 yang murah, bermanfaat, dan menarik</t>
+          <t>7 manfaat baby oil untuk wajah serta cara menggunakannya dengan aman</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 11:09:39 +0700</t>
+          <t>Sun, 02 Aug 2026 11:14:29 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Menjelang peringatan HUT ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026, berbagai lingkungan mulai ...</t>
+          <t>Baby oil tidak hanya digunakan untuk perawatan kulit bayi, tetapi juga kerap dimanfaatkan sebagai bagian dari rutinitas ...</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676419/20-ide-hadiah-lomba-17-agustus-2026-yang-murah-bermanfaat-dan-menarik</t>
+          <t>https://www.antaranews.com/berita/5676420/7-manfaat-baby-oil-untuk-wajah-serta-cara-menggunakannya-dengan-aman</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2025/08/17/pesta-rakyat-hut-ri-di-monas-2602245.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/23/Tua.jpg</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1448,28 +1448,28 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Kenapa badan sakit-sakit setelah gym? Ini sebab dan cara atasinya</t>
+          <t>20 ide hadiah lomba 17 Agustus 2026 yang murah, bermanfaat, dan menarik</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 10:38:58 +0700</t>
+          <t>Sun, 02 Aug 2026 11:09:39 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Merasa badan pegal atau sakit-sakit setelah berolahraga di gym merupakan hal yang umum dialami, terutama oleh pemula ...</t>
+          <t>Menjelang peringatan HUT ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026, berbagai lingkungan mulai ...</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676396/kenapa-badan-sakit-sakit-setelah-gym-ini-sebab-dan-cara-atasinya</t>
+          <t>https://www.antaranews.com/berita/5676419/20-ide-hadiah-lomba-17-agustus-2026-yang-murah-bermanfaat-dan-menarik</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/03/02/indeks-pembangunan-manusia-kalimantan-barat-2670125.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/08/17/pesta-rakyat-hut-ri-di-monas-2602245.jpg</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1486,28 +1486,28 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10 tanda tubuh kekurangan air yang sering diabaikan</t>
+          <t>Kenapa badan sakit-sakit setelah gym? Ini sebab dan cara atasinya</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 10:04:12 +0700</t>
+          <t>Sun, 02 Aug 2026 10:38:58 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Air merupakan komponen utama dalam tubuh manusia yang berperan penting dalam menjaga suhu tubuh, melancarkan sirkulasi ...</t>
+          <t>Merasa badan pegal atau sakit-sakit setelah berolahraga di gym merupakan hal yang umum dialami, terutama oleh pemula ...</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676363/10-tanda-tubuh-kekurangan-air-yang-sering-diabaikan</t>
+          <t>https://www.antaranews.com/berita/5676396/kenapa-badan-sakit-sakit-setelah-gym-ini-sebab-dan-cara-atasinya</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/03/04/Aqua-pic.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/02/indeks-pembangunan-manusia-kalimantan-barat-2670125.jpg</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1524,28 +1524,28 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10 barang wajib dibawa saat liburan agar perjalanan nyaman dan praktis</t>
+          <t>10 tanda tubuh kekurangan air yang sering diabaikan</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 10:00:42 +0700</t>
+          <t>Sun, 02 Aug 2026 10:04:12 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Liburan menjadi momen yang dinantikan banyak orang untuk melepas penat dari rutinitas sehari-hari. Namun, perjalanan ...</t>
+          <t>Air merupakan komponen utama dalam tubuh manusia yang berperan penting dalam menjaga suhu tubuh, melancarkan sirkulasi ...</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676355/10-barang-wajib-dibawa-saat-liburan-agar-perjalanan-nyaman-dan-praktis</t>
+          <t>https://www.antaranews.com/berita/5676363/10-tanda-tubuh-kekurangan-air-yang-sering-diabaikan</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/1000887286.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/04/Aqua-pic.jpg</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1562,28 +1562,28 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>10 cara mengatur keuangan bulanan agar gaji tidak cepat habis</t>
+          <t>10 barang wajib dibawa saat liburan agar perjalanan nyaman dan praktis</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 09:54:58 +0700</t>
+          <t>Sun, 02 Aug 2026 10:00:42 +0700</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Mengelola keuangan bulanan menjadi tantangan bagi banyak orang, terutama saat pengeluaran terasa lebih besar daripada ...</t>
+          <t>Liburan menjadi momen yang dinantikan banyak orang untuk melepas penat dari rutinitas sehari-hari. Namun, perjalanan ...</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676352/10-cara-mengatur-keuangan-bulanan-agar-gaji-tidak-cepat-habis</t>
+          <t>https://www.antaranews.com/berita/5676355/10-barang-wajib-dibawa-saat-liburan-agar-perjalanan-nyaman-dan-praktis</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/09/Ilustrasi-mengatur-keuangan.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/1000887286.jpg</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1595,33 +1595,33 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>tekno</t>
+          <t>lifestyle</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>10 cara mengurangi screen time agar mata tetap sehat dan tidur nyenyak</t>
+          <t>10 cara mengatur keuangan bulanan agar gaji tidak cepat habis</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 10:13:01 +0700</t>
+          <t>Sun, 02 Aug 2026 09:54:58 +0700</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Penggunaan ponsel, tablet, dan komputer telah menjadi bagian dari kehidupan sehari-hari. Mulai dari bekerja, belajar, ...</t>
+          <t>Mengelola keuangan bulanan menjadi tantangan bagi banyak orang, terutama saat pengeluaran terasa lebih besar daripada ...</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676376/10-cara-mengurangi-screen-time-agar-mata-tetap-sehat-dan-tidur-nyenyak</t>
+          <t>https://www.antaranews.com/berita/5676352/10-cara-mengatur-keuangan-bulanan-agar-gaji-tidak-cepat-habis</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/09/CDAD3117-892E-4E7F-AF44-CF43EED7F052.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/09/Ilustrasi-mengatur-keuangan.jpg</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1638,28 +1638,28 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Cara tepat restart paksa iPhone yang error agar kembali normal</t>
+          <t>10 cara mengurangi screen time agar mata tetap sehat dan tidur nyenyak</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 10:09:15 +0700</t>
+          <t>Sun, 02 Aug 2026 10:13:01 +0700</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>iPhone yang tiba-tiba error, layar tidak merespons sentuhan, atau berhenti di logo Apple menjadi masalah yang cukup ...</t>
+          <t>Penggunaan ponsel, tablet, dan komputer telah menjadi bagian dari kehidupan sehari-hari. Mulai dari bekerja, belajar, ...</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676373/cara-tepat-restart-paksa-iphone-yang-error-agar-kembali-normal</t>
+          <t>https://www.antaranews.com/berita/5676376/10-cara-mengurangi-screen-time-agar-mata-tetap-sehat-dan-tidur-nyenyak</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/13/InShot_20260513_153025843.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/09/CDAD3117-892E-4E7F-AF44-CF43EED7F052.jpeg</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1671,33 +1671,33 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>photo</t>
+          <t>tekno</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Andi Sultan raih medali emas Asian Taekwondo Indonesia Open Championships</t>
+          <t>Cara tepat restart paksa iPhone yang error agar kembali normal</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 21:13:46 +0700</t>
+          <t>Sun, 02 Aug 2026 10:09:15 +0700</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Atlet Taekwondo Indonesia Andi Sultan mengibarkan bendera Merah Putih usai memenangkan pertandingan final nomor Poomsae Freestyle Individual Men Over 17 pada 8th Asian Taekwondo Indonesia Open Championships 2026 di Tennis Indoor Senayan, Jakarta, Minggu (2/8/2026). Andi Sultan meraih medali emas dengan perolehan skor 8.540 poin. ANTARA FOTO/Dhemas Reviyanto/sgd</t>
+          <t>iPhone yang tiba-tiba error, layar tidak merespons sentuhan, atau berhenti di logo Apple menjadi masalah yang cukup ...</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/foto/5676816/andi-sultan-raih-medali-emas-asian-taekwondo-indonesia-open-championships</t>
+          <t>https://www.antaranews.com/berita/5676373/cara-tepat-restart-paksa-iphone-yang-error-agar-kembali-normal</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/255x170/2026/08/02/andi-sultan-raih-medali-emas-asian-taekwondo-indonesia-open-championships-2026-020826-dr-03.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/13/InShot_20260513_153025843.jpg</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1714,28 +1714,28 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Latihan Timnas Indonesia jelang lawan Vietnam</t>
+          <t>Andi Sultan raih medali emas Asian Taekwondo Indonesia Open Championships</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 21:09:02 +0700</t>
+          <t>Sun, 02 Aug 2026 21:13:46 +0700</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Sejumlah pesepak bola Timnas Indonesia mengikuti sesi latihan di Stadion GBK, Jakarta, Minggu (2/8/2026). Latihan Timnas Indonesia untuk persiapan laga ketiga Grup A Piala AFF 2026 melawan Vietnam di Stadion Pakansari pada Senin (3/8/2026). ANTARA FOTO/Fakhri Hermansyah/sgd</t>
+          <t>Atlet Taekwondo Indonesia Andi Sultan mengibarkan bendera Merah Putih usai memenangkan pertandingan final nomor Poomsae Freestyle Individual Men Over 17 pada 8th Asian Taekwondo Indonesia Open Championships 2026 di Tennis Indoor Senayan, Jakarta, Minggu (2/8/2026). Andi Sultan meraih medali emas dengan perolehan skor 8.540 poin. ANTARA FOTO/Dhemas Reviyanto/sgd</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/foto/5676812/latihan-timnas-indonesia-jelang-lawan-vietnam</t>
+          <t>https://www.antaranews.com/foto/5676816/andi-sultan-raih-medali-emas-asian-taekwondo-indonesia-open-championships</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/255x170/2026/08/02/Latihan-Timnas-Indonesia-jelang-melawan-Vietnam-020826-Fah-4.jpg</t>
+          <t>https://cdn.antaranews.com/cache/255x170/2026/08/02/andi-sultan-raih-medali-emas-asian-taekwondo-indonesia-open-championships-2026-020826-dr-03.jpg</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1752,28 +1752,28 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>KMP Mutiara Sentosa 2 terbakar di perairan Sumenep</t>
+          <t>Latihan Timnas Indonesia jelang lawan Vietnam</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 19:00:25 +0700</t>
+          <t>Sun, 02 Aug 2026 21:09:02 +0700</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Kapal Mutiara Sentosa 2 terbakar di perairan Sumenep, Jawa Timur, Minggu (2/8/2026). Kapal Motor Penumpang (KMP) Mutiara Sentosa 2 yang berpenumpang sekitar 250 orang penumpang tersebut mengalami kebakaran saat melakukan pelayaran dari Surabaya ke Makassar. ANTARAFOTO/Umarul Faruq/sgd</t>
+          <t>Sejumlah pesepak bola Timnas Indonesia mengikuti sesi latihan di Stadion GBK, Jakarta, Minggu (2/8/2026). Latihan Timnas Indonesia untuk persiapan laga ketiga Grup A Piala AFF 2026 melawan Vietnam di Stadion Pakansari pada Senin (3/8/2026). ANTARA FOTO/Fakhri Hermansyah/sgd</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/foto/5676725/kmp-mutiara-sentosa-2-terbakar-di-perairan-sumenep</t>
+          <t>https://www.antaranews.com/foto/5676812/latihan-timnas-indonesia-jelang-lawan-vietnam</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/255x170/2026/08/02/KMP-Mutiara-Sentosa-2-terbakar-di-Sumenep-02082026-Um-9.jpg</t>
+          <t>https://cdn.antaranews.com/cache/255x170/2026/08/02/Latihan-Timnas-Indonesia-jelang-melawan-Vietnam-020826-Fah-4.jpg</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1790,28 +1790,28 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Melihat balap babi di Amerika</t>
+          <t>KMP Mutiara Sentosa 2 terbakar di perairan Sumenep</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 17:06:31 +0700</t>
+          <t>Sun, 02 Aug 2026 19:00:25 +0700</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Sejumlah babi berlomba dalam kompetisi balap babi pada Orange County Fair di Costa Mesa, California, Amerika Serikat, (1/8/2026). ANTARA FOTO/Xinhua/Qiu Chen/sgd</t>
+          <t>Kapal Mutiara Sentosa 2 terbakar di perairan Sumenep, Jawa Timur, Minggu (2/8/2026). Kapal Motor Penumpang (KMP) Mutiara Sentosa 2 yang berpenumpang sekitar 250 orang penumpang tersebut mengalami kebakaran saat melakukan pelayaran dari Surabaya ke Makassar. ANTARAFOTO/Umarul Faruq/sgd</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/foto/5676656/melihat-balap-babi-di-amerika</t>
+          <t>https://www.antaranews.com/foto/5676725/kmp-mutiara-sentosa-2-terbakar-di-perairan-sumenep</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/255x170/2026/08/02/XxjpbeE000086_20260802_PEPFN0A001.jpg</t>
+          <t>https://cdn.antaranews.com/cache/255x170/2026/08/02/KMP-Mutiara-Sentosa-2-terbakar-di-Sumenep-02082026-Um-9.jpg</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">

</xml_diff>